<commit_message>
commit the documentation change 2
commit the documentation change 2
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\4eme\T4\TPI\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5C1BDC-0F22-4548-924C-A64DFA0DEE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6124FC-C879-4CB0-9B80-EA196355E5D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="54">
   <si>
     <t>Jour</t>
   </si>
@@ -186,6 +186,21 @@
   </si>
   <si>
     <t>Rédaction rapport — section Conception (stratégie de test)</t>
+  </si>
+  <si>
+    <t>Création de l'environement de travail et création du repository</t>
+  </si>
+  <si>
+    <t>création l'environement sur Clion avec Plateformio (plusieurs installation) + création du répository et upload de tous les fichier du dossier local de l'analyse et de la conception</t>
+  </si>
+  <si>
+    <t>Brasure des éléments éléctronique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai pu braser les éléments j'ai eu juste un soucis de brasure avec le ring. 2 pistes se sont arracher pendant que j'essayais de en réarranger la brasure selon un autre enseignant M. Favre pourrais reussir a réavoir les 2 éléments </t>
+  </si>
+  <si>
+    <t>Rendu 3 au chef de projet et aux 2 Expert</t>
   </si>
 </sst>
 </file>
@@ -910,7 +925,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -925,7 +940,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.75</c:v>
+                  <c:v>2.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2085,7 +2100,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>46136</v>
       </c>
@@ -2105,7 +2120,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>46136</v>
       </c>
@@ -2343,29 +2358,65 @@
       </c>
       <c r="F20" s="17"/>
     </row>
-    <row r="21" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="6"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="17"/>
-    </row>
-    <row r="22" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="17"/>
+    <row r="21" spans="1:6" ht="51.75" x14ac:dyDescent="0.3">
+      <c r="A21" s="6">
+        <v>46140</v>
+      </c>
+      <c r="B21" s="14">
+        <v>2</v>
+      </c>
+      <c r="C21" s="11">
+        <v>1</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="51.75" x14ac:dyDescent="0.3">
+      <c r="A22" s="6">
+        <v>46140</v>
+      </c>
+      <c r="B22" s="14">
+        <v>2</v>
+      </c>
+      <c r="C22" s="11">
+        <v>2</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="17"/>
+      <c r="A23" s="6">
+        <v>46140</v>
+      </c>
+      <c r="B23" s="14">
+        <v>2</v>
+      </c>
+      <c r="C23" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
@@ -6261,7 +6312,7 @@
       </c>
       <c r="B4" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6306,7 +6357,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>1.75</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Push for the 4rd checkup with th work of Thursday and Friday
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6124FC-C879-4CB0-9B80-EA196355E5D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71D7014-46B5-4D3B-B2D8-E2DB0BC8196E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="68">
   <si>
     <t>Jour</t>
   </si>
@@ -201,6 +201,53 @@
   </si>
   <si>
     <t>Rendu 3 au chef de projet et aux 2 Expert</t>
+  </si>
+  <si>
+    <t>Montage de tous les composant sur la bread board avec l'arduino</t>
+  </si>
+  <si>
+    <t>Sauf le ring</t>
+  </si>
+  <si>
+    <t>Brasure du ring cassé pour tester</t>
+  </si>
+  <si>
+    <t>Programmation pour test</t>
+  </si>
+  <si>
+    <t>Programmation assisté par IA juste pour les test afin de diagnostiquer les porblème le plutôt possible</t>
+  </si>
+  <si>
+    <t>Effectue les test et comprendre les soucis</t>
+  </si>
+  <si>
+    <t>Teste de tous les éléments et essai de ressoudre ou de comprendre pourquoi cela ne fonctionne pas j'ai pu ainsi faire fonctionner le BME680, j'ai découvert que le RTC DS1307 ne pouvais pas fonctionner sans pile donc impossible de le tester pour le moment, les bouton fonctionne sans aucun problème avec l'anti-bounce, l'affichage 14 segment a 1 segement mort sur chacun des 2 premier digit et le ring ne fonctionne toujours pas</t>
+  </si>
+  <si>
+    <t>Discussion avec Chef de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discussion avec M.Favre :
+- Ring mort ou alors voir avec lui pour la réparation : M. Favre a fourni 2 nouveau quart de ring qui étais mort
+- Affichage 14 segments sur les 2 premier caractère la bar verticale en bas a droite ne s'allume pas : M. Favre va fournir un nouveau 14 segment prochainement eet analyser de son coté pourquoi celui-ci a 2 segement cassé
+- Documentation conception : M. Favre est d'accord que j'avance sur la réalisation surtout en temps de test de fonctionnement
+- pile CR1220 : M. Favre va fournir une pile lundi il n'avais pas prévu cet eventualité et vu que c'est un format très spécifique nous en avons pas en stock
+- Retour projet : M. Favre n'a pas eu le temps de lire la doc nous prendrons le temps Lundi </t>
+  </si>
+  <si>
+    <t>Brasure du ring avec les nouveau quart en remplacement</t>
+  </si>
+  <si>
+    <t>Test du ring</t>
+  </si>
+  <si>
+    <t>quelque complication durant le test mais maintenant 1/2 du ring s'allume</t>
+  </si>
+  <si>
+    <t>Rendu 4 au chef de projet et aux 2 Expert</t>
+  </si>
+  <si>
+    <t>Mise a jour des fichier PDF, Actualisation du Repository et Rédaction du mail et envoi</t>
   </si>
 </sst>
 </file>
@@ -925,10 +972,10 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3</c:v>
+                  <c:v>9.25</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>9.25</c:v>
@@ -940,7 +987,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.25</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1956,7 +2003,7 @@
     <col min="2" max="2" width="13.375" style="15" customWidth="1"/>
     <col min="3" max="3" width="15.25" style="12" customWidth="1"/>
     <col min="4" max="4" width="24.75" style="5" customWidth="1"/>
-    <col min="5" max="5" width="68.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="70.25" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="85.625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2406,7 +2453,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="11">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>13</v>
@@ -2419,89 +2466,172 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="17"/>
+      <c r="A24" s="6">
+        <v>46142</v>
+      </c>
+      <c r="B24" s="14">
+        <v>2</v>
+      </c>
+      <c r="C24" s="11">
+        <v>1.25</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="6"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="8"/>
+      <c r="A25" s="6">
+        <v>46142</v>
+      </c>
+      <c r="B25" s="14">
+        <v>2</v>
+      </c>
+      <c r="C25" s="11">
+        <v>2</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>56</v>
+      </c>
       <c r="F25" s="17"/>
     </row>
-    <row r="26" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="17"/>
-    </row>
-    <row r="27" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="6"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="17"/>
-    </row>
-    <row r="28" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="6"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="17"/>
+    <row r="26" spans="1:6" ht="34.5" x14ac:dyDescent="0.3">
+      <c r="A26" s="6">
+        <v>46142</v>
+      </c>
+      <c r="B26" s="14">
+        <v>2</v>
+      </c>
+      <c r="C26" s="11">
+        <v>1</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="103.5" x14ac:dyDescent="0.3">
+      <c r="A27" s="6">
+        <v>46142</v>
+      </c>
+      <c r="B27" s="14">
+        <v>2</v>
+      </c>
+      <c r="C27" s="12">
+        <v>3</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="207" x14ac:dyDescent="0.3">
+      <c r="A28" s="6">
+        <v>46143</v>
+      </c>
+      <c r="B28" s="14">
+        <v>2</v>
+      </c>
+      <c r="C28" s="11">
+        <v>1</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="6"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="8"/>
+      <c r="A29" s="6">
+        <v>46143</v>
+      </c>
+      <c r="B29" s="14">
+        <v>2</v>
+      </c>
+      <c r="C29" s="11">
+        <v>2</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="F29" s="17"/>
     </row>
     <row r="30" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="6"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="17"/>
-    </row>
-    <row r="31" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="6"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="17"/>
+      <c r="A30" s="6">
+        <v>46143</v>
+      </c>
+      <c r="B30" s="14">
+        <v>2</v>
+      </c>
+      <c r="C30" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6">
+        <v>46143</v>
+      </c>
+      <c r="B31" s="14">
+        <v>2</v>
+      </c>
+      <c r="C31" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="6"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="11"/>
       <c r="D32" s="7"/>
       <c r="E32" s="8"/>
       <c r="F32" s="17"/>
     </row>
     <row r="33" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="6"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="11"/>
       <c r="D33" s="7"/>
       <c r="E33" s="8"/>
       <c r="F33" s="17"/>
     </row>
     <row r="34" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="11"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
       <c r="F34" s="17"/>
@@ -6236,11 +6366,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B300" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B35:B300 B1:B31" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C300" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C26 C35:C300 C28:C31" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
       <formula1>0.25</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -6312,7 +6442,7 @@
       </c>
       <c r="B4" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>3</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6321,7 +6451,7 @@
       </c>
       <c r="B5" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6357,7 +6487,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>2.25</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>